<commit_message>
Data source updates and verification.
</commit_message>
<xml_diff>
--- a/data/docs/data_sources.xlsx
+++ b/data/docs/data_sources.xlsx
@@ -591,11 +591,11 @@
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
     <col width="60" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="51" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
     <col width="60" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -722,7 +722,11 @@
       <c r="D3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>The downloaded dataset has the same number of freguesias (3,092) as reported in the original Gouveia et al. (2019) article. Gouveia et al. (2019) explicitly cite the 2016 CAOP Portugal map. The downloaded geometry was visually inspected and compared to the plots in the article; no discrepancies were found.</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>https://www.dgterritorio.gov.pt/cartografia/cartografia-tematica/caop</t>
@@ -730,7 +734,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>CAOP 2016 freguesia boundaries | 2016 shapefiles for continental Portugal and all its parts:
+          <t>Versões anteriores -&gt; 2016 -&gt; shapefiles for continental Portugal, Madeira, and three Açores parts:
 https://www.dgterritorio.gov.pt/cartografia/cartografia-tematica/caop</t>
         </is>
       </c>
@@ -763,16 +767,12 @@
           <t>2023-10-31</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>Additional source metadata:
-- provider: Direção-Geral do Território
-- evidence_ids: ["manual_inspection"]
-- local_artifacts: [""]
-- usage_status: pipeline_input</t>
-        </is>
-      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>E:\energy_povert_from_space_data\data\CAOP_2016_shapefiles</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -793,11 +793,7 @@
       <c r="D4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Download lineage supplied and verified by the user; not independent verification of citations or pipeline transformations.</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>https://ec.europa.eu/eurostat/web/nuts/local-administrative-units</t>
@@ -805,27 +801,48 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Eurostat LAU to NUTS correspondence | https://ec.europa.eu/eurostat/web/nuts/local-administrative-units</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>LAU – NUTS 2016, EU-28 and EFTA / available candidate countries (2017).</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Eurostat. (2017). LAU – NUTS 2016, EU-28 and EFTA / available candidate countries [Data set]. https://ec.europa.eu/eurostat/web/nuts/local-administrative-units</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>Additional source metadata:
-- evidence_ids: ["download_notes"]
-- local_artifacts: ["data/adm_maps/freguesias_to_NUTS3.csv"]
-- usage_status: pipeline_input</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Freguesias are grouped spatially by NUTS3 to prevent spatial leakage in the analysis. The correspondence is used to aggregate the CAOP 2016 freguesia geometries to NUTS3 regions.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>LAU – NUTS 2016, EU-28 and EFTA / available candidate countries (2017)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>E:\git_projects\energy_poverty_from_space\data\adm_maps\freguesias_to_NUTS3.csv</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -863,13 +880,17 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Elvidge, C. D., Ghosh, T., Hsu, F.-C., Zhizhin, M., &amp; Taneja, J. (2021). Annual global VIIRS nighttime lights datasets for 2015–2020. Remote Sensing, 13(5), 922.</t>
+          <t>Elvidge, C. D., Zhizhin, M., Ghosh, T., Hsu, F.-C., &amp; Taneja, J. (2021). Annual time series of global VIIRS nighttime lights derived from monthly averages: 2012 to 2019. *Remote Sensing, 13*(5), 922. https://doi.org/10.3390/rs13050922</t>
         </is>
       </c>
       <c r="I5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Precedence in the literature for using VIIRS night-time lights as a proxy for settlement and socioeconomic activity.</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
           <t>VNL v2.1</t>

</xml_diff>